<commit_message>
20260818 commit : temp, early
</commit_message>
<xml_diff>
--- a/ppt, excel, script/최종/01_3조_딱코_AI_드론 기반 보행자 검색추적을 위한 실시간 관제 시스템_1차프로젝트산출물/02_3조_딱코_AI_드론 기반 보행자 검색추적을 위한 실시간 관제 시스템_요구사항명세서.xlsx
+++ b/ppt, excel, script/최종/01_3조_딱코_AI_드론 기반 보행자 검색추적을 위한 실시간 관제 시스템_1차프로젝트산출물/02_3조_딱코_AI_드론 기반 보행자 검색추적을 위한 실시간 관제 시스템_요구사항명세서.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lyh\first_1_pjt\pjt_first\ppt, excel, script\최종\01_3조_딱코_AI_드론 기반 보행자 검색추적을 위한 실시간 관제 시스템_1차프로젝트산출물\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DW\Desktop\01_3조_딱코_AI_드론 기반 보행자 검색추적을 위한 실시간 관제 시스템_1차프로젝트산출물\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7995"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12285"/>
   </bookViews>
   <sheets>
     <sheet name="요구사항" sheetId="2" r:id="rId1"/>

</xml_diff>